<commit_message>
Ajuste en farmatodo para que lea correctamente los importes del remittance sin importar formato, y ajuste en funcion diferencias en entorno de pruebas. Esto hizo que se deba ajustar los entornos de prueba
</commit_message>
<xml_diff>
--- a/Pruebas/Archivos/Template/Colombia/Template_HRC_Jeronimo.xlsx
+++ b/Pruebas/Archivos/Template/Colombia/Template_HRC_Jeronimo.xlsx
@@ -583,7 +583,7 @@
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>16/12/2025</t>
+          <t>19/12/2025</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -4750,7 +4750,7 @@
       </c>
       <c r="G199" s="10" t="inlineStr">
         <is>
-          <t>CSR</t>
+          <t>WOB</t>
         </is>
       </c>
       <c r="H199" s="6" t="n">

</xml_diff>